<commit_message>
Added raw yield sheets to spreadsheets
</commit_message>
<xml_diff>
--- a/Data/1999_F105_CO_AGIIS/1999_F105_CO_AGIIS_Yield_Quality.xlsx
+++ b/Data/1999_F105_CO_AGIIS/1999_F105_CO_AGIIS_Yield_Quality.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26626"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\mnt\Data1\USDA-ALARC\GIS\PDI tool\tool\Data\1999_F105_CO_AGIIS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\mnt\Data1\USDA-ALARC\GIS\PDI project\cottondata\Data\1999_F105_CO_AGIIS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D86A293E-7BE4-425D-8D22-7F1F53517155}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27C37EDD-8560-401D-853B-3B37D98F2C3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-4590" yWindow="-28920" windowWidth="18240" windowHeight="29040" xr2:uid="{5485CBB2-C13A-4C0B-BAC8-38661C175E52}"/>
+    <workbookView xWindow="16410" yWindow="-22920" windowWidth="17715" windowHeight="17625" xr2:uid="{5485CBB2-C13A-4C0B-BAC8-38661C175E52}"/>
   </bookViews>
   <sheets>
     <sheet name="Raw Scale" sheetId="1" r:id="rId1"/>
     <sheet name="Plot Scale" sheetId="2" r:id="rId2"/>
     <sheet name="Compare" sheetId="3" r:id="rId3"/>
+    <sheet name="RawData" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="169">
   <si>
     <t>Column</t>
   </si>
@@ -428,6 +429,123 @@
   </si>
   <si>
     <t>p16S</t>
+  </si>
+  <si>
+    <t>wn</t>
+  </si>
+  <si>
+    <t>wN</t>
+  </si>
+  <si>
+    <t>Wn</t>
+  </si>
+  <si>
+    <t>WN</t>
+  </si>
+  <si>
+    <t>average</t>
+  </si>
+  <si>
+    <t>21/22</t>
+  </si>
+  <si>
+    <t>bag 7 &amp;8</t>
+  </si>
+  <si>
+    <t>19/20</t>
+  </si>
+  <si>
+    <t>bag 5&amp;6</t>
+  </si>
+  <si>
+    <t>17/18</t>
+  </si>
+  <si>
+    <t>bag 3 &amp;4</t>
+  </si>
+  <si>
+    <t>15/16</t>
+  </si>
+  <si>
+    <t>bag 1 &amp;2</t>
+  </si>
+  <si>
+    <t>Lint</t>
+  </si>
+  <si>
+    <t>Plot#</t>
+  </si>
+  <si>
+    <t>Assume35%</t>
+  </si>
+  <si>
+    <t>Pure Lint wt (g)</t>
+  </si>
+  <si>
+    <t>Seed wt (g)</t>
+  </si>
+  <si>
+    <t>Sub sample wt (g)</t>
+  </si>
+  <si>
+    <t>Total Sample wt(kg)</t>
+  </si>
+  <si>
+    <t>South</t>
+  </si>
+  <si>
+    <t>North</t>
+  </si>
+  <si>
+    <t>Plot #</t>
+  </si>
+  <si>
+    <t>Plot Averages</t>
+  </si>
+  <si>
+    <t>Percent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Sample Row</t>
+  </si>
+  <si>
+    <t>Calculated</t>
+  </si>
+  <si>
+    <t>Two 44 m2 areas harvested per plot (north &amp; south)</t>
+  </si>
+  <si>
+    <t>2 rows (2m) by 22 m lengths (44 sq m)</t>
+  </si>
+  <si>
+    <t>Area Harvestd:</t>
+  </si>
+  <si>
+    <t>2.92 kg</t>
+  </si>
+  <si>
+    <t>Bucket wt:</t>
+  </si>
+  <si>
+    <t>0.51 kg</t>
+  </si>
+  <si>
+    <t>Bag wt :</t>
+  </si>
+  <si>
+    <t>Date of Processing</t>
+  </si>
+  <si>
+    <t>November 12 1999</t>
+  </si>
+  <si>
+    <t>Date of Harvest</t>
+  </si>
+  <si>
+    <t>Final Harvest/ Processing</t>
+  </si>
+  <si>
+    <t>LiMIE Cotton 1999                      Final Harvest</t>
   </si>
 </sst>
 </file>
@@ -441,7 +559,7 @@
     <numFmt numFmtId="166" formatCode="mm/dd/yyyy"/>
     <numFmt numFmtId="167" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -462,8 +580,22 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -476,8 +608,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="15"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="13"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -494,12 +638,125 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="14" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
@@ -517,10 +774,78 @@
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="167" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" xfId="4" applyFont="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="4" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" xfId="4" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="2" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="16" fontId="4" fillId="0" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="2" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="2" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="2" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="2" quotePrefix="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="2" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="2" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="5">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Comma 2" xfId="3" xr:uid="{B1C561A0-89BE-4D89-8C32-1BB2A5D16A28}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="2" xr:uid="{13735EA2-FD8C-47EA-BE47-7B22F4FE0C32}"/>
+    <cellStyle name="Percent 2" xfId="4" xr:uid="{C5D9AEB1-8BBE-4FDC-908A-9AB12848217B}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -3111,9 +3436,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -3151,7 +3476,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -3257,7 +3582,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -3399,7 +3724,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -3408,99 +3733,99 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4D7E8EA-A5C9-47F2-8D6E-B68B0450AD04}">
   <dimension ref="A1:AE59"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="5" max="5" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="8.88671875" customWidth="1"/>
+    <col min="5" max="5" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="8.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="18" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="19" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A19">
         <f>22*1.016*2</f>
         <v>44.704000000000001</v>
@@ -3509,7 +3834,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="20" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>10000</v>
       </c>
@@ -3520,7 +3845,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="22" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:31" x14ac:dyDescent="0.25">
       <c r="C22" s="1"/>
       <c r="D22" s="1" t="s">
         <v>2</v>
@@ -3601,7 +3926,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="23" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:31" x14ac:dyDescent="0.25">
       <c r="C23" s="1"/>
       <c r="D23" s="1"/>
       <c r="E23" s="1"/>
@@ -3613,7 +3938,7 @@
       <c r="O23" s="1"/>
       <c r="P23" s="1"/>
     </row>
-    <row r="24" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:31" x14ac:dyDescent="0.25">
       <c r="C24" s="1"/>
       <c r="D24" s="1"/>
       <c r="E24" s="1"/>
@@ -3649,7 +3974,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="25" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>0</v>
       </c>
@@ -3735,7 +4060,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="26" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:31" x14ac:dyDescent="0.25">
       <c r="C26" s="1"/>
       <c r="D26" s="1"/>
       <c r="E26" s="1"/>
@@ -3803,7 +4128,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="27" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>0</v>
       </c>
@@ -3868,7 +4193,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="28" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>1</v>
       </c>
@@ -3978,7 +4303,7 @@
         <v>3250.8031757286672</v>
       </c>
     </row>
-    <row r="29" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>1</v>
       </c>
@@ -4045,7 +4370,7 @@
       <c r="AD29" s="4"/>
       <c r="AE29" s="4"/>
     </row>
-    <row r="30" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>2</v>
       </c>
@@ -4155,7 +4480,7 @@
         <v>3038.7405235672413</v>
       </c>
     </row>
-    <row r="31" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>2</v>
       </c>
@@ -4222,7 +4547,7 @@
       <c r="AD31" s="4"/>
       <c r="AE31" s="4"/>
     </row>
-    <row r="32" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>3</v>
       </c>
@@ -4332,7 +4657,7 @@
         <v>3136.3754230945283</v>
       </c>
     </row>
-    <row r="33" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>3</v>
       </c>
@@ -4399,7 +4724,7 @@
       <c r="AD33" s="4"/>
       <c r="AE33" s="4"/>
     </row>
-    <row r="34" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>4</v>
       </c>
@@ -4509,7 +4834,7 @@
         <v>3700.9226102566799</v>
       </c>
     </row>
-    <row r="35" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>4</v>
       </c>
@@ -4576,7 +4901,7 @@
       <c r="AD35" s="4"/>
       <c r="AE35" s="4"/>
     </row>
-    <row r="36" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>1</v>
       </c>
@@ -4686,7 +5011,7 @@
         <v>3301.2221315009056</v>
       </c>
     </row>
-    <row r="37" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>1</v>
       </c>
@@ -4753,7 +5078,7 @@
       <c r="AD37" s="4"/>
       <c r="AE37" s="4"/>
     </row>
-    <row r="38" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>2</v>
       </c>
@@ -4863,7 +5188,7 @@
         <v>3489.5680683002138</v>
       </c>
     </row>
-    <row r="39" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>2</v>
       </c>
@@ -4930,7 +5255,7 @@
       <c r="AD39" s="4"/>
       <c r="AE39" s="4"/>
     </row>
-    <row r="40" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>3</v>
       </c>
@@ -5040,7 +5365,7 @@
         <v>2877.3269336497351</v>
       </c>
     </row>
-    <row r="41" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>3</v>
       </c>
@@ -5107,7 +5432,7 @@
       <c r="AD41" s="4"/>
       <c r="AE41" s="4"/>
     </row>
-    <row r="42" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>4</v>
       </c>
@@ -5217,7 +5542,7 @@
         <v>3457.7500615552799</v>
       </c>
     </row>
-    <row r="43" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>4</v>
       </c>
@@ -5284,7 +5609,7 @@
       <c r="AD43" s="4"/>
       <c r="AE43" s="4"/>
     </row>
-    <row r="44" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>1</v>
       </c>
@@ -5394,7 +5719,7 @@
         <v>3906.3058658136788</v>
       </c>
     </row>
-    <row r="45" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>1</v>
       </c>
@@ -5461,7 +5786,7 @@
       <c r="AD45" s="4"/>
       <c r="AE45" s="4"/>
     </row>
-    <row r="46" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>2</v>
       </c>
@@ -5571,7 +5896,7 @@
         <v>3255.0806469525633</v>
       </c>
     </row>
-    <row r="47" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>2</v>
       </c>
@@ -5638,7 +5963,7 @@
       <c r="AD47" s="4"/>
       <c r="AE47" s="4"/>
     </row>
-    <row r="48" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>3</v>
       </c>
@@ -5748,7 +6073,7 @@
         <v>3376.4006950039693</v>
       </c>
     </row>
-    <row r="49" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>3</v>
       </c>
@@ -5815,7 +6140,7 @@
       <c r="AD49" s="4"/>
       <c r="AE49" s="4"/>
     </row>
-    <row r="50" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>4</v>
       </c>
@@ -5925,7 +6250,7 @@
         <v>3151.9424549082414</v>
       </c>
     </row>
-    <row r="51" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>4</v>
       </c>
@@ -5992,7 +6317,7 @@
       <c r="AD51" s="4"/>
       <c r="AE51" s="4"/>
     </row>
-    <row r="52" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>1</v>
       </c>
@@ -6102,7 +6427,7 @@
         <v>3131.1834754370207</v>
       </c>
     </row>
-    <row r="53" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>1</v>
       </c>
@@ -6169,7 +6494,7 @@
       <c r="AD53" s="4"/>
       <c r="AE53" s="4"/>
     </row>
-    <row r="54" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>2</v>
       </c>
@@ -6279,7 +6604,7 @@
         <v>3055.5296136522757</v>
       </c>
     </row>
-    <row r="55" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>2</v>
       </c>
@@ -6346,7 +6671,7 @@
       <c r="AD55" s="4"/>
       <c r="AE55" s="4"/>
     </row>
-    <row r="56" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>3</v>
       </c>
@@ -6456,7 +6781,7 @@
         <v>3404.4632895018776</v>
       </c>
     </row>
-    <row r="57" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>3</v>
       </c>
@@ -6523,7 +6848,7 @@
       <c r="AD57" s="4"/>
       <c r="AE57" s="4"/>
     </row>
-    <row r="58" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>4</v>
       </c>
@@ -6609,7 +6934,7 @@
         <v>3104.0516075471201</v>
       </c>
     </row>
-    <row r="59" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>4</v>
       </c>
@@ -6679,12 +7004,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02F174ED-B270-4962-A7F2-21DE7C85D8A3}">
   <dimension ref="A1:N22"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="1"/>
       <c r="B1" s="1" t="s">
         <v>2</v>
@@ -6726,7 +7051,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -6738,7 +7063,7 @@
       <c r="M2" s="1"/>
       <c r="N2" s="1"/>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -6762,7 +7087,7 @@
       <c r="M3" s="1"/>
       <c r="N3" s="1"/>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>59</v>
       </c>
@@ -6803,7 +7128,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
@@ -6839,7 +7164,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>59</v>
       </c>
@@ -6875,7 +7200,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
         <v>82</v>
       </c>
@@ -6919,7 +7244,7 @@
         <v>3250.8031757286672</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
         <v>83</v>
       </c>
@@ -6963,7 +7288,7 @@
         <v>3038.7405235672413</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
         <v>84</v>
       </c>
@@ -7007,7 +7332,7 @@
         <v>3136.3754230945283</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
         <v>85</v>
       </c>
@@ -7051,7 +7376,7 @@
         <v>3700.9226102566799</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
         <v>86</v>
       </c>
@@ -7095,7 +7420,7 @@
         <v>3301.2221315009056</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
         <v>87</v>
       </c>
@@ -7139,7 +7464,7 @@
         <v>3489.5680683002138</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
         <v>88</v>
       </c>
@@ -7183,7 +7508,7 @@
         <v>2877.3269336497351</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
         <v>89</v>
       </c>
@@ -7227,7 +7552,7 @@
         <v>3457.7500615552799</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
         <v>90</v>
       </c>
@@ -7271,7 +7596,7 @@
         <v>3906.3058658136788</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
         <v>91</v>
       </c>
@@ -7315,7 +7640,7 @@
         <v>3255.0806469525633</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
         <v>92</v>
       </c>
@@ -7359,7 +7684,7 @@
         <v>3376.4006950039693</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A18" s="14" t="s">
         <v>93</v>
       </c>
@@ -7403,7 +7728,7 @@
         <v>3151.9424549082414</v>
       </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
         <v>94</v>
       </c>
@@ -7447,7 +7772,7 @@
         <v>3131.1834754370207</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A20" s="14" t="s">
         <v>95</v>
       </c>
@@ -7491,7 +7816,7 @@
         <v>3055.5296136522757</v>
       </c>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A21" s="14" t="s">
         <v>96</v>
       </c>
@@ -7535,7 +7860,7 @@
         <v>3404.4632895018776</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A22" s="14" t="s">
         <v>97</v>
       </c>
@@ -7587,9 +7912,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C33FAA98-8EB4-4946-B5DF-4604489C86BA}">
   <dimension ref="A1:N36"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
         <v>77</v>
       </c>
@@ -7597,7 +7922,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>80</v>
       </c>
@@ -7608,12 +7933,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="N3">
         <v>3000</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>35</v>
       </c>
@@ -7624,7 +7949,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -7635,7 +7960,7 @@
         <v>1211.5332121190984</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -7646,7 +7971,7 @@
         <v>1313.1449604474033</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -7657,7 +7982,7 @@
         <v>1360.1641147774778</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -7668,7 +7993,7 @@
         <v>1098.3951659392242</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>5</v>
       </c>
@@ -7679,7 +8004,7 @@
         <v>1156.362001113592</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -7690,7 +8015,7 @@
         <v>1319.4700820282728</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -7701,7 +8026,7 @@
         <v>1446.0731514336503</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -7712,7 +8037,7 @@
         <v>1512.1844234228763</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -7723,7 +8048,7 @@
         <v>1296.6009654062752</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>12</v>
       </c>
@@ -7734,7 +8059,7 @@
         <v>1304.0369925502048</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>13</v>
       </c>
@@ -7745,7 +8070,7 @@
         <v>1359.7643245292779</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>14</v>
       </c>
@@ -7756,7 +8081,7 @@
         <v>1391.7670584149178</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>15</v>
       </c>
@@ -7767,7 +8092,7 @@
         <v>1180.5215518134178</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>16</v>
       </c>
@@ -7778,7 +8103,7 @@
         <v>1076.8347697178133</v>
       </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>17</v>
       </c>
@@ -7789,7 +8114,7 @@
         <v>1344.2063668744433</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>18</v>
       </c>
@@ -7800,7 +8125,7 @@
         <v>1418.8882541151193</v>
       </c>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>19</v>
       </c>
@@ -7811,7 +8136,7 @@
         <v>1488.6073117936467</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>20</v>
       </c>
@@ -7822,7 +8147,7 @@
         <v>1632.0689468557202</v>
       </c>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>21</v>
       </c>
@@ -7833,7 +8158,7 @@
         <v>1192.0471876877571</v>
       </c>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>22</v>
       </c>
@@ -7844,7 +8169,7 @@
         <v>1347.7752753239677</v>
       </c>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>23</v>
       </c>
@@ -7858,7 +8183,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>24</v>
       </c>
@@ -7872,7 +8197,7 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>25</v>
       </c>
@@ -7883,7 +8208,7 @@
         <v>1069.390402075227</v>
       </c>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>26</v>
       </c>
@@ -7894,7 +8219,7 @@
         <v>1327.9636104943193</v>
       </c>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>27</v>
       </c>
@@ -7905,7 +8230,7 @@
         <v>1227.6899640436568</v>
       </c>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>28</v>
       </c>
@@ -7916,7 +8241,7 @@
         <v>1252.5060731244787</v>
       </c>
     </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>29</v>
       </c>
@@ -7927,7 +8252,7 @@
         <v>1175.5400674477182</v>
       </c>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>30</v>
       </c>
@@ -7938,7 +8263,7 @@
         <v>1205.4998349262246</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>31</v>
       </c>
@@ -7949,7 +8274,7 @@
         <v>1415.417684308243</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>32</v>
       </c>
@@ -7960,7 +8285,7 @@
         <v>1311.2085376334057</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>33</v>
       </c>
@@ -7971,7 +8296,7 @@
         <v>614.35847516545289</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>34</v>
       </c>
@@ -7986,4 +8311,2390 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89DCD964-CE2E-42B2-8832-9F76AF57831E}">
+  <dimension ref="A1:S73"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="19.140625" style="15" customWidth="1"/>
+    <col min="2" max="3" width="9.140625" style="15"/>
+    <col min="4" max="4" width="15.85546875" style="15" customWidth="1"/>
+    <col min="5" max="5" width="15.5703125" style="15" customWidth="1"/>
+    <col min="6" max="6" width="10.28515625" style="15" customWidth="1"/>
+    <col min="7" max="7" width="13.42578125" style="15" customWidth="1"/>
+    <col min="8" max="9" width="9.140625" style="15"/>
+    <col min="10" max="10" width="13" style="15" customWidth="1"/>
+    <col min="11" max="11" width="12.28515625" style="15" customWidth="1"/>
+    <col min="12" max="14" width="9.140625" style="15"/>
+    <col min="15" max="15" width="14.28515625" style="15" customWidth="1"/>
+    <col min="16" max="16" width="13.28515625" style="15" customWidth="1"/>
+    <col min="17" max="16384" width="9.140625" style="15"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:19" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A1" s="45" t="s">
+        <v>168</v>
+      </c>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="46" t="s">
+        <v>167</v>
+      </c>
+      <c r="E1" s="45"/>
+      <c r="F1" s="45"/>
+      <c r="G1" s="45"/>
+    </row>
+    <row r="2" spans="1:19" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A2" s="46" t="s">
+        <v>166</v>
+      </c>
+      <c r="B2" s="45" t="s">
+        <v>165</v>
+      </c>
+      <c r="D2" s="45"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="45"/>
+    </row>
+    <row r="3" spans="1:19" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A3" s="47" t="s">
+        <v>164</v>
+      </c>
+      <c r="B3" s="45"/>
+      <c r="C3" s="45"/>
+      <c r="D3" s="45"/>
+      <c r="E3" s="45"/>
+      <c r="F3" s="45"/>
+      <c r="G3" s="45"/>
+    </row>
+    <row r="4" spans="1:19" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A4" s="46" t="s">
+        <v>163</v>
+      </c>
+      <c r="B4" s="45" t="s">
+        <v>162</v>
+      </c>
+      <c r="C4" s="45"/>
+      <c r="D4" s="45"/>
+      <c r="E4" s="45"/>
+      <c r="F4" s="45"/>
+      <c r="G4" s="45"/>
+    </row>
+    <row r="5" spans="1:19" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A5" s="45" t="s">
+        <v>161</v>
+      </c>
+      <c r="B5" s="45" t="s">
+        <v>160</v>
+      </c>
+      <c r="C5" s="45"/>
+      <c r="D5" s="45"/>
+      <c r="E5" s="45"/>
+      <c r="F5" s="45"/>
+      <c r="G5" s="45"/>
+    </row>
+    <row r="6" spans="1:19" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A6" s="45" t="s">
+        <v>159</v>
+      </c>
+      <c r="B6" s="46" t="s">
+        <v>158</v>
+      </c>
+      <c r="C6" s="45"/>
+      <c r="D6" s="45"/>
+      <c r="E6" s="45"/>
+      <c r="F6" s="45"/>
+      <c r="G6" s="45"/>
+    </row>
+    <row r="7" spans="1:19" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A7" s="45"/>
+      <c r="B7" s="46" t="s">
+        <v>157</v>
+      </c>
+      <c r="C7" s="45"/>
+      <c r="D7" s="45"/>
+      <c r="E7" s="45"/>
+      <c r="F7" s="45"/>
+      <c r="G7" s="45"/>
+    </row>
+    <row r="8" spans="1:19" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A8" s="45"/>
+      <c r="B8" s="45"/>
+      <c r="C8" s="45"/>
+      <c r="D8" s="45"/>
+      <c r="E8" s="45"/>
+      <c r="F8" s="45"/>
+      <c r="G8" s="45"/>
+    </row>
+    <row r="9" spans="1:19" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="16"/>
+      <c r="B9" s="16"/>
+      <c r="C9" s="16"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="16"/>
+      <c r="F9" s="16"/>
+      <c r="G9" s="16"/>
+      <c r="H9" s="44" t="s">
+        <v>156</v>
+      </c>
+      <c r="I9" s="44"/>
+      <c r="J9" s="44"/>
+      <c r="K9" s="44"/>
+    </row>
+    <row r="10" spans="1:19" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="16"/>
+      <c r="B10" s="43" t="s">
+        <v>155</v>
+      </c>
+      <c r="C10" s="42"/>
+      <c r="D10" s="41"/>
+      <c r="E10" s="41"/>
+      <c r="F10" s="41"/>
+      <c r="G10" s="41"/>
+      <c r="H10" s="31" t="s">
+        <v>154</v>
+      </c>
+      <c r="I10" s="31" t="s">
+        <v>154</v>
+      </c>
+      <c r="J10" s="31"/>
+      <c r="K10" s="31"/>
+      <c r="M10" s="40" t="s">
+        <v>153</v>
+      </c>
+      <c r="N10" s="40"/>
+      <c r="O10" s="40"/>
+      <c r="P10" s="40"/>
+    </row>
+    <row r="11" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="39" t="s">
+        <v>152</v>
+      </c>
+      <c r="B11" s="38" t="s">
+        <v>151</v>
+      </c>
+      <c r="C11" s="38" t="s">
+        <v>150</v>
+      </c>
+      <c r="D11" s="37" t="s">
+        <v>149</v>
+      </c>
+      <c r="E11" s="36" t="s">
+        <v>148</v>
+      </c>
+      <c r="F11" s="36" t="s">
+        <v>147</v>
+      </c>
+      <c r="G11" s="35" t="s">
+        <v>146</v>
+      </c>
+      <c r="H11" s="34" t="s">
+        <v>49</v>
+      </c>
+      <c r="I11" s="33" t="s">
+        <v>143</v>
+      </c>
+      <c r="J11" s="32" t="s">
+        <v>78</v>
+      </c>
+      <c r="K11" s="32" t="s">
+        <v>79</v>
+      </c>
+      <c r="L11" s="18" t="s">
+        <v>145</v>
+      </c>
+      <c r="M11" s="31" t="s">
+        <v>144</v>
+      </c>
+      <c r="N11" s="31" t="s">
+        <v>143</v>
+      </c>
+      <c r="O11" s="31" t="s">
+        <v>78</v>
+      </c>
+      <c r="P11" s="31" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="12" spans="1:19" ht="15" x14ac:dyDescent="0.25">
+      <c r="A12" s="29">
+        <v>1</v>
+      </c>
+      <c r="B12" s="29" t="s">
+        <v>142</v>
+      </c>
+      <c r="C12" s="29"/>
+      <c r="D12" s="30">
+        <f>8.56 +7.12</f>
+        <v>15.68</v>
+      </c>
+      <c r="E12" s="30">
+        <f>1211.8-64.82</f>
+        <v>1146.98</v>
+      </c>
+      <c r="F12" s="29">
+        <f>648.44-23.95</f>
+        <v>624.49</v>
+      </c>
+      <c r="G12" s="29">
+        <f>454.76-64.82</f>
+        <v>389.94</v>
+      </c>
+      <c r="H12" s="21">
+        <f>F12/E12</f>
+        <v>0.54446459397722713</v>
+      </c>
+      <c r="I12" s="20">
+        <f>G12/E12</f>
+        <v>0.33997105442117559</v>
+      </c>
+      <c r="J12" s="18">
+        <f>D12*H12/44*10000</f>
+        <v>1940.273825809755</v>
+      </c>
+      <c r="K12" s="18">
+        <f>I12*D12/44*10000</f>
+        <v>1211.5332121190984</v>
+      </c>
+      <c r="L12" s="18">
+        <f>D12/44*10000*0.35</f>
+        <v>1247.2727272727273</v>
+      </c>
+      <c r="M12" s="15">
+        <f>A12</f>
+        <v>1</v>
+      </c>
+      <c r="N12" s="19">
+        <f>AVERAGE(I12:I13)</f>
+        <v>0.33765348501582793</v>
+      </c>
+      <c r="O12" s="17">
+        <f>AVERAGE(J12:J13)</f>
+        <v>2040.2336305224117</v>
+      </c>
+      <c r="P12" s="17">
+        <f>AVERAGE(K12:K13)</f>
+        <v>1262.3390862832507</v>
+      </c>
+      <c r="R12" s="17">
+        <f>SUM(O12:P12)</f>
+        <v>3302.5727168056624</v>
+      </c>
+      <c r="S12" s="17">
+        <f>SUM(O12:P12)</f>
+        <v>3302.5727168056624</v>
+      </c>
+    </row>
+    <row r="13" spans="1:19" ht="15" x14ac:dyDescent="0.25">
+      <c r="A13" s="22">
+        <v>1</v>
+      </c>
+      <c r="B13" s="22"/>
+      <c r="C13" s="22" t="s">
+        <v>141</v>
+      </c>
+      <c r="D13" s="22">
+        <f>9.39+7.84</f>
+        <v>17.23</v>
+      </c>
+      <c r="E13" s="22">
+        <f>1203.35-64.82</f>
+        <v>1138.53</v>
+      </c>
+      <c r="F13" s="22">
+        <f>646.2-23.95</f>
+        <v>622.25</v>
+      </c>
+      <c r="G13" s="22">
+        <f>446.61-64.82</f>
+        <v>381.79</v>
+      </c>
+      <c r="H13" s="21">
+        <f>F13/E13</f>
+        <v>0.5465380798046604</v>
+      </c>
+      <c r="I13" s="20">
+        <f>G13/E13</f>
+        <v>0.33533591561048021</v>
+      </c>
+      <c r="J13" s="18">
+        <f>D13*H13/44*10000</f>
+        <v>2140.1934352350681</v>
+      </c>
+      <c r="K13" s="18">
+        <f>I13*D13/44*10000</f>
+        <v>1313.1449604474033</v>
+      </c>
+      <c r="L13" s="18">
+        <f>D13/44*10000*0.35</f>
+        <v>1370.5681818181818</v>
+      </c>
+      <c r="N13" s="19"/>
+      <c r="R13" s="17"/>
+      <c r="S13" s="17">
+        <f>SUM(O14:P14)</f>
+        <v>3091.7113358374359</v>
+      </c>
+    </row>
+    <row r="14" spans="1:19" ht="15" x14ac:dyDescent="0.25">
+      <c r="A14" s="22">
+        <v>2</v>
+      </c>
+      <c r="B14" s="28" t="s">
+        <v>140</v>
+      </c>
+      <c r="C14" s="22"/>
+      <c r="D14" s="27">
+        <f>11+5.38</f>
+        <v>16.38</v>
+      </c>
+      <c r="E14" s="22">
+        <f>1107.66-64.82</f>
+        <v>1042.8400000000001</v>
+      </c>
+      <c r="F14" s="22">
+        <f>606.22-23.95</f>
+        <v>582.27</v>
+      </c>
+      <c r="G14" s="22">
+        <f>445.84-64.82</f>
+        <v>381.02</v>
+      </c>
+      <c r="H14" s="21">
+        <f>F14/E14</f>
+        <v>0.55835027425108352</v>
+      </c>
+      <c r="I14" s="20">
+        <f>G14/E14</f>
+        <v>0.36536764987917603</v>
+      </c>
+      <c r="J14" s="18">
+        <f>D14*H14/44*10000</f>
+        <v>2078.5857936892608</v>
+      </c>
+      <c r="K14" s="18">
+        <f>I14*D14/44*10000</f>
+        <v>1360.1641147774778</v>
+      </c>
+      <c r="L14" s="18">
+        <f>D14/44*10000*0.35</f>
+        <v>1302.9545454545453</v>
+      </c>
+      <c r="M14" s="15">
+        <f>A14</f>
+        <v>2</v>
+      </c>
+      <c r="N14" s="19">
+        <f>AVERAGE(I14:I15)</f>
+        <v>0.35678104144292322</v>
+      </c>
+      <c r="O14" s="17">
+        <f>AVERAGE(J14:J15)</f>
+        <v>1862.4316954790847</v>
+      </c>
+      <c r="P14" s="17">
+        <f>AVERAGE(K14:K15)</f>
+        <v>1229.2796403583511</v>
+      </c>
+      <c r="R14" s="17">
+        <f>SUM(O14:P14)</f>
+        <v>3091.7113358374359</v>
+      </c>
+      <c r="S14" s="17">
+        <f>SUM(O16:P16)</f>
+        <v>3194.1456598409109</v>
+      </c>
+    </row>
+    <row r="15" spans="1:19" ht="15" x14ac:dyDescent="0.25">
+      <c r="A15" s="22">
+        <v>2</v>
+      </c>
+      <c r="B15" s="22"/>
+      <c r="C15" s="22" t="s">
+        <v>139</v>
+      </c>
+      <c r="D15" s="22">
+        <f>4.45+9.43</f>
+        <v>13.879999999999999</v>
+      </c>
+      <c r="E15" s="22">
+        <f>1036.26-64.82</f>
+        <v>971.44</v>
+      </c>
+      <c r="F15" s="22">
+        <f>530.92-23.95</f>
+        <v>506.96999999999997</v>
+      </c>
+      <c r="G15" s="22">
+        <f>403.07-64.82</f>
+        <v>338.25</v>
+      </c>
+      <c r="H15" s="21">
+        <f>F15/E15</f>
+        <v>0.52187474265008638</v>
+      </c>
+      <c r="I15" s="20">
+        <f>G15/E15</f>
+        <v>0.34819443300667047</v>
+      </c>
+      <c r="J15" s="18">
+        <f>D15*H15/44*10000</f>
+        <v>1646.2775972689087</v>
+      </c>
+      <c r="K15" s="18">
+        <f>I15*D15/44*10000</f>
+        <v>1098.3951659392242</v>
+      </c>
+      <c r="L15" s="18">
+        <f>D15/44*10000*0.35</f>
+        <v>1104.090909090909</v>
+      </c>
+      <c r="N15" s="19"/>
+      <c r="R15" s="17"/>
+      <c r="S15" s="17">
+        <f>SUM(O18:P18)</f>
+        <v>3757.3062651339719</v>
+      </c>
+    </row>
+    <row r="16" spans="1:19" ht="15" x14ac:dyDescent="0.25">
+      <c r="A16" s="22">
+        <v>3</v>
+      </c>
+      <c r="B16" s="22" t="s">
+        <v>138</v>
+      </c>
+      <c r="C16" s="22"/>
+      <c r="D16" s="22">
+        <f>8.38+6.43</f>
+        <v>14.81</v>
+      </c>
+      <c r="E16" s="22">
+        <f>1073.84-64.82</f>
+        <v>1009.02</v>
+      </c>
+      <c r="F16" s="22">
+        <f>564.09-23.95</f>
+        <v>540.14</v>
+      </c>
+      <c r="G16" s="22">
+        <f>411.47-64.82</f>
+        <v>346.65000000000003</v>
+      </c>
+      <c r="H16" s="21">
+        <f>F16/E16</f>
+        <v>0.53531149035698</v>
+      </c>
+      <c r="I16" s="20">
+        <f>G16/E16</f>
+        <v>0.34355116846048644</v>
+      </c>
+      <c r="J16" s="18">
+        <f>D16*H16/44*10000</f>
+        <v>1801.8098118606531</v>
+      </c>
+      <c r="K16" s="18">
+        <f>I16*D16/44*10000</f>
+        <v>1156.362001113592</v>
+      </c>
+      <c r="L16" s="18">
+        <f>D16/44*10000*0.35</f>
+        <v>1178.0681818181818</v>
+      </c>
+      <c r="M16" s="15">
+        <f>A16</f>
+        <v>3</v>
+      </c>
+      <c r="N16" s="19">
+        <f>AVERAGE(I16:I17)</f>
+        <v>0.34632965401149396</v>
+      </c>
+      <c r="O16" s="17">
+        <f>AVERAGE(J16:J17)</f>
+        <v>1956.2296182699783</v>
+      </c>
+      <c r="P16" s="17">
+        <f>AVERAGE(K16:K17)</f>
+        <v>1237.9160415709325</v>
+      </c>
+      <c r="R16" s="17">
+        <f>SUM(O16:P16)</f>
+        <v>3194.1456598409109</v>
+      </c>
+      <c r="S16" s="17">
+        <f>SUM(O20:P20)</f>
+        <v>3357.49740135293</v>
+      </c>
+    </row>
+    <row r="17" spans="1:19" ht="15" x14ac:dyDescent="0.25">
+      <c r="A17" s="22">
+        <v>3</v>
+      </c>
+      <c r="B17" s="22"/>
+      <c r="C17" s="22" t="s">
+        <v>137</v>
+      </c>
+      <c r="D17" s="22">
+        <f>10.26+6.37</f>
+        <v>16.63</v>
+      </c>
+      <c r="E17" s="22">
+        <f>906.88-64.82</f>
+        <v>842.06</v>
+      </c>
+      <c r="F17" s="22">
+        <f>494.19-23.95</f>
+        <v>470.24</v>
+      </c>
+      <c r="G17" s="22">
+        <f>358.79-64.82</f>
+        <v>293.97000000000003</v>
+      </c>
+      <c r="H17" s="21">
+        <f>F17/E17</f>
+        <v>0.55844001615086813</v>
+      </c>
+      <c r="I17" s="20">
+        <f>G17/E17</f>
+        <v>0.34910813956250153</v>
+      </c>
+      <c r="J17" s="18">
+        <f>D17*H17/44*10000</f>
+        <v>2110.6494246793036</v>
+      </c>
+      <c r="K17" s="18">
+        <f>I17*D17/44*10000</f>
+        <v>1319.4700820282728</v>
+      </c>
+      <c r="L17" s="18">
+        <f>D17/44*10000*0.35</f>
+        <v>1322.840909090909</v>
+      </c>
+      <c r="N17" s="19"/>
+      <c r="R17" s="17"/>
+      <c r="S17" s="17">
+        <f>SUM(O22:P22)</f>
+        <v>3544.7784091200569</v>
+      </c>
+    </row>
+    <row r="18" spans="1:19" ht="15" x14ac:dyDescent="0.25">
+      <c r="A18" s="22">
+        <v>4</v>
+      </c>
+      <c r="B18" s="22" t="s">
+        <v>136</v>
+      </c>
+      <c r="C18" s="22"/>
+      <c r="D18" s="22">
+        <f>6.95+11.1</f>
+        <v>18.05</v>
+      </c>
+      <c r="E18" s="22">
+        <f>1262.05-64.82</f>
+        <v>1197.23</v>
+      </c>
+      <c r="F18" s="22">
+        <f>679.56-23.95</f>
+        <v>655.6099999999999</v>
+      </c>
+      <c r="G18" s="22">
+        <f>486.85-64.82</f>
+        <v>422.03000000000003</v>
+      </c>
+      <c r="H18" s="21">
+        <f>F18/E18</f>
+        <v>0.54760572321107881</v>
+      </c>
+      <c r="I18" s="20">
+        <f>G18/E18</f>
+        <v>0.35250536655446324</v>
+      </c>
+      <c r="J18" s="18">
+        <f>D18*H18/44*10000</f>
+        <v>2246.4280236272671</v>
+      </c>
+      <c r="K18" s="18">
+        <f>I18*D18/44*10000</f>
+        <v>1446.0731514336503</v>
+      </c>
+      <c r="L18" s="18">
+        <f>D18/44*10000*0.35</f>
+        <v>1435.7954545454543</v>
+      </c>
+      <c r="M18" s="15">
+        <f>A18</f>
+        <v>4</v>
+      </c>
+      <c r="N18" s="19">
+        <f>AVERAGE(I18:I19)</f>
+        <v>0.35283472847523201</v>
+      </c>
+      <c r="O18" s="17">
+        <f>AVERAGE(J18:J19)</f>
+        <v>2278.1774777057085</v>
+      </c>
+      <c r="P18" s="17">
+        <f>AVERAGE(K18:K19)</f>
+        <v>1479.1287874282634</v>
+      </c>
+      <c r="R18" s="17">
+        <f>SUM(O18:P18)</f>
+        <v>3757.3062651339719</v>
+      </c>
+      <c r="S18" s="17">
+        <f>SUM(O24:P24)</f>
+        <v>2927.9721625087886</v>
+      </c>
+    </row>
+    <row r="19" spans="1:19" ht="15" x14ac:dyDescent="0.25">
+      <c r="A19" s="22">
+        <v>4</v>
+      </c>
+      <c r="B19" s="22"/>
+      <c r="C19" s="22" t="s">
+        <v>135</v>
+      </c>
+      <c r="D19" s="22">
+        <f>9.36+9.48</f>
+        <v>18.84</v>
+      </c>
+      <c r="E19" s="22">
+        <f>933-64.82</f>
+        <v>868.18000000000006</v>
+      </c>
+      <c r="F19" s="22">
+        <f>492.31-23.95</f>
+        <v>468.36</v>
+      </c>
+      <c r="G19" s="22">
+        <f>371.43-64.82</f>
+        <v>306.61</v>
+      </c>
+      <c r="H19" s="21">
+        <f>F19/E19</f>
+        <v>0.539473381096086</v>
+      </c>
+      <c r="I19" s="20">
+        <f>G19/E19</f>
+        <v>0.35316409039600083</v>
+      </c>
+      <c r="J19" s="18">
+        <f>D19*H19/44*10000</f>
+        <v>2309.9269317841499</v>
+      </c>
+      <c r="K19" s="18">
+        <f>I19*D19/44*10000</f>
+        <v>1512.1844234228763</v>
+      </c>
+      <c r="L19" s="18">
+        <f>D19/44*10000*0.35</f>
+        <v>1498.6363636363635</v>
+      </c>
+      <c r="N19" s="19"/>
+      <c r="R19" s="17"/>
+      <c r="S19" s="17">
+        <f>SUM(O26:P26)</f>
+        <v>3513.189047249406</v>
+      </c>
+    </row>
+    <row r="20" spans="1:19" ht="15" x14ac:dyDescent="0.25">
+      <c r="A20" s="22">
+        <v>5</v>
+      </c>
+      <c r="B20" s="22">
+        <v>23</v>
+      </c>
+      <c r="C20" s="22"/>
+      <c r="D20" s="22">
+        <v>16.53</v>
+      </c>
+      <c r="E20" s="22">
+        <f>1181.26-64.82</f>
+        <v>1116.44</v>
+      </c>
+      <c r="F20" s="22">
+        <f>632.4-23.95</f>
+        <v>608.44999999999993</v>
+      </c>
+      <c r="G20" s="22">
+        <f>450.14-64.82</f>
+        <v>385.32</v>
+      </c>
+      <c r="H20" s="21">
+        <f>F20/E20</f>
+        <v>0.54499122209881401</v>
+      </c>
+      <c r="I20" s="20">
+        <f>G20/E20</f>
+        <v>0.34513274336283184</v>
+      </c>
+      <c r="J20" s="18">
+        <f>D20*H20/44*10000</f>
+        <v>2047.4329321121356</v>
+      </c>
+      <c r="K20" s="18">
+        <f>I20*D20/44*10000</f>
+        <v>1296.6009654062752</v>
+      </c>
+      <c r="L20" s="18">
+        <f>D20/44*10000*0.35</f>
+        <v>1314.8863636363637</v>
+      </c>
+      <c r="M20" s="15">
+        <f>A20</f>
+        <v>5</v>
+      </c>
+      <c r="N20" s="19">
+        <f>AVERAGE(I20:I21)</f>
+        <v>0.34781874697832804</v>
+      </c>
+      <c r="O20" s="17">
+        <f>AVERAGE(J20:J21)</f>
+        <v>2057.1784223746899</v>
+      </c>
+      <c r="P20" s="17">
+        <f>AVERAGE(K20:K21)</f>
+        <v>1300.31897897824</v>
+      </c>
+      <c r="R20" s="17">
+        <f>SUM(O20:P20)</f>
+        <v>3357.49740135293</v>
+      </c>
+      <c r="S20" s="17">
+        <f>SUM(O28:P28)</f>
+        <v>3968.5824027610593</v>
+      </c>
+    </row>
+    <row r="21" spans="1:19" ht="15" x14ac:dyDescent="0.25">
+      <c r="A21" s="22">
+        <v>5</v>
+      </c>
+      <c r="B21" s="22"/>
+      <c r="C21" s="22">
+        <v>28</v>
+      </c>
+      <c r="D21" s="22">
+        <v>16.37</v>
+      </c>
+      <c r="E21" s="22">
+        <f>940.5-64.82</f>
+        <v>875.68000000000006</v>
+      </c>
+      <c r="F21" s="22">
+        <f>510.44-23.95</f>
+        <v>486.49</v>
+      </c>
+      <c r="G21" s="22">
+        <f>371.75-64.82</f>
+        <v>306.93</v>
+      </c>
+      <c r="H21" s="21">
+        <f>F21/E21</f>
+        <v>0.55555682441074361</v>
+      </c>
+      <c r="I21" s="20">
+        <f>G21/E21</f>
+        <v>0.35050475059382419</v>
+      </c>
+      <c r="J21" s="18">
+        <f>D21*H21/44*10000</f>
+        <v>2066.923912637244</v>
+      </c>
+      <c r="K21" s="18">
+        <f>I21*D21/44*10000</f>
+        <v>1304.0369925502048</v>
+      </c>
+      <c r="L21" s="18">
+        <f>D21/44*10000*0.35</f>
+        <v>1302.1590909090908</v>
+      </c>
+      <c r="N21" s="19"/>
+      <c r="R21" s="17"/>
+      <c r="S21" s="17">
+        <f>SUM(O30:P30)</f>
+        <v>3302.4388617654195</v>
+      </c>
+    </row>
+    <row r="22" spans="1:19" ht="15" x14ac:dyDescent="0.25">
+      <c r="A22" s="22">
+        <v>6</v>
+      </c>
+      <c r="B22" s="22">
+        <v>24</v>
+      </c>
+      <c r="C22" s="22"/>
+      <c r="D22" s="22">
+        <v>17.3</v>
+      </c>
+      <c r="E22" s="22">
+        <f>1091-64.82</f>
+        <v>1026.18</v>
+      </c>
+      <c r="F22" s="22">
+        <f>595.24-23.95</f>
+        <v>571.29</v>
+      </c>
+      <c r="G22" s="22">
+        <f>419.71-64.82</f>
+        <v>354.89</v>
+      </c>
+      <c r="H22" s="21">
+        <f>F22/E22</f>
+        <v>0.55671519616441556</v>
+      </c>
+      <c r="I22" s="20">
+        <f>G22/E22</f>
+        <v>0.34583601317507645</v>
+      </c>
+      <c r="J22" s="18">
+        <f>D22*H22/44*10000</f>
+        <v>2188.9029303737252</v>
+      </c>
+      <c r="K22" s="18">
+        <f>I22*D22/44*10000</f>
+        <v>1359.7643245292779</v>
+      </c>
+      <c r="L22" s="18">
+        <f>D22/44*10000*0.35</f>
+        <v>1376.1363636363635</v>
+      </c>
+      <c r="M22" s="15">
+        <f>A22</f>
+        <v>6</v>
+      </c>
+      <c r="N22" s="19">
+        <f>AVERAGE(I22:I23)</f>
+        <v>0.35093472336153936</v>
+      </c>
+      <c r="O22" s="17">
+        <f>AVERAGE(J22:J23)</f>
+        <v>2169.0127176479591</v>
+      </c>
+      <c r="P22" s="17">
+        <f>AVERAGE(K22:K23)</f>
+        <v>1375.7656914720978</v>
+      </c>
+      <c r="R22" s="17">
+        <f>SUM(O22:P22)</f>
+        <v>3544.7784091200569</v>
+      </c>
+      <c r="S22" s="17">
+        <f>SUM(O32:P32)</f>
+        <v>3430.6151684361776</v>
+      </c>
+    </row>
+    <row r="23" spans="1:19" ht="15" x14ac:dyDescent="0.25">
+      <c r="A23" s="22">
+        <v>6</v>
+      </c>
+      <c r="B23" s="22"/>
+      <c r="C23" s="22">
+        <v>29</v>
+      </c>
+      <c r="D23" s="22">
+        <v>17.2</v>
+      </c>
+      <c r="E23" s="22">
+        <f>1305.5-64.83</f>
+        <v>1240.67</v>
+      </c>
+      <c r="F23" s="22">
+        <f>706.04-23.95</f>
+        <v>682.08999999999992</v>
+      </c>
+      <c r="G23" s="22">
+        <f>506.54-64.82</f>
+        <v>441.72</v>
+      </c>
+      <c r="H23" s="21">
+        <f>F23/E23</f>
+        <v>0.54977552451497969</v>
+      </c>
+      <c r="I23" s="20">
+        <f>G23/E23</f>
+        <v>0.35603343354800226</v>
+      </c>
+      <c r="J23" s="18">
+        <f>D23*H23/44*10000</f>
+        <v>2149.122504922193</v>
+      </c>
+      <c r="K23" s="18">
+        <f>I23*D23/44*10000</f>
+        <v>1391.7670584149178</v>
+      </c>
+      <c r="L23" s="18">
+        <f>D23/44*10000*0.35</f>
+        <v>1368.181818181818</v>
+      </c>
+      <c r="N23" s="19"/>
+      <c r="R23" s="17"/>
+      <c r="S23" s="17">
+        <f>SUM(O34:P34)</f>
+        <v>3208.4730965116482</v>
+      </c>
+    </row>
+    <row r="24" spans="1:19" ht="15" x14ac:dyDescent="0.25">
+      <c r="A24" s="22">
+        <v>7</v>
+      </c>
+      <c r="B24" s="22">
+        <v>26</v>
+      </c>
+      <c r="C24" s="22"/>
+      <c r="D24" s="22">
+        <v>14.92</v>
+      </c>
+      <c r="E24" s="22">
+        <f>1030.4-64.82</f>
+        <v>965.58000000000015</v>
+      </c>
+      <c r="F24" s="22">
+        <f>555.96-23.95</f>
+        <v>532.01</v>
+      </c>
+      <c r="G24" s="22">
+        <f>400.98-64.82</f>
+        <v>336.16</v>
+      </c>
+      <c r="H24" s="21">
+        <f>F24/E24</f>
+        <v>0.55097454379751021</v>
+      </c>
+      <c r="I24" s="20">
+        <f>G24/E24</f>
+        <v>0.3481430849851902</v>
+      </c>
+      <c r="J24" s="18">
+        <f>D24*H24/44*10000</f>
+        <v>1868.3045894224665</v>
+      </c>
+      <c r="K24" s="18">
+        <f>I24*D24/44*10000</f>
+        <v>1180.5215518134178</v>
+      </c>
+      <c r="L24" s="18">
+        <f>D24/44*10000*0.35</f>
+        <v>1186.8181818181818</v>
+      </c>
+      <c r="M24" s="15">
+        <f>A24</f>
+        <v>7</v>
+      </c>
+      <c r="N24" s="19">
+        <f>AVERAGE(I24:I25)</f>
+        <v>0.34268623953025978</v>
+      </c>
+      <c r="O24" s="17">
+        <f>AVERAGE(J24:J25)</f>
+        <v>1799.2940017431733</v>
+      </c>
+      <c r="P24" s="17">
+        <f>AVERAGE(K24:K25)</f>
+        <v>1128.6781607656155</v>
+      </c>
+      <c r="R24" s="17">
+        <f>SUM(O24:P24)</f>
+        <v>2927.9721625087886</v>
+      </c>
+      <c r="S24" s="17">
+        <f>SUM(O36:P36)</f>
+        <v>3181.5701850390869</v>
+      </c>
+    </row>
+    <row r="25" spans="1:19" ht="15" x14ac:dyDescent="0.25">
+      <c r="A25" s="22">
+        <v>7</v>
+      </c>
+      <c r="B25" s="22"/>
+      <c r="C25" s="22">
+        <v>30</v>
+      </c>
+      <c r="D25" s="22">
+        <v>14.05</v>
+      </c>
+      <c r="E25" s="22">
+        <f>1268.6-64.82</f>
+        <v>1203.78</v>
+      </c>
+      <c r="F25" s="22">
+        <f>676.24-23.95</f>
+        <v>652.29</v>
+      </c>
+      <c r="G25" s="22">
+        <f>470.78-64.83</f>
+        <v>405.95</v>
+      </c>
+      <c r="H25" s="21">
+        <f>F25/E25</f>
+        <v>0.54186811543637536</v>
+      </c>
+      <c r="I25" s="20">
+        <f>G25/E25</f>
+        <v>0.33722939407532937</v>
+      </c>
+      <c r="J25" s="18">
+        <f>D25*H25/44*10000</f>
+        <v>1730.2834140638804</v>
+      </c>
+      <c r="K25" s="18">
+        <f>I25*D25/44*10000</f>
+        <v>1076.8347697178133</v>
+      </c>
+      <c r="L25" s="18">
+        <f>D25/44*10000*0.35</f>
+        <v>1117.6136363636365</v>
+      </c>
+      <c r="N25" s="19"/>
+      <c r="R25" s="17"/>
+      <c r="S25" s="17">
+        <f>SUM(O38:P38)</f>
+        <v>3096.8891681623718</v>
+      </c>
+    </row>
+    <row r="26" spans="1:19" ht="15" x14ac:dyDescent="0.25">
+      <c r="A26" s="22">
+        <v>8</v>
+      </c>
+      <c r="B26" s="22">
+        <v>27</v>
+      </c>
+      <c r="C26" s="22"/>
+      <c r="D26" s="22">
+        <v>16.89</v>
+      </c>
+      <c r="E26" s="22">
+        <f>1142.9-64.82</f>
+        <v>1078.0800000000002</v>
+      </c>
+      <c r="F26" s="22">
+        <f>611.3-23.95</f>
+        <v>587.34999999999991</v>
+      </c>
+      <c r="G26" s="22">
+        <f>442.34-64.82</f>
+        <v>377.52</v>
+      </c>
+      <c r="H26" s="21">
+        <f>F26/E26</f>
+        <v>0.54481114574057565</v>
+      </c>
+      <c r="I26" s="20">
+        <f>G26/E26</f>
+        <v>0.35017809439002667</v>
+      </c>
+      <c r="J26" s="18">
+        <f>D26*H26/44*10000</f>
+        <v>2091.3318753541644</v>
+      </c>
+      <c r="K26" s="18">
+        <f>I26*D26/44*10000</f>
+        <v>1344.2063668744433</v>
+      </c>
+      <c r="L26" s="18">
+        <f>D26/44*10000*0.35</f>
+        <v>1343.5227272727273</v>
+      </c>
+      <c r="M26" s="15">
+        <f>A26</f>
+        <v>8</v>
+      </c>
+      <c r="N26" s="19">
+        <f>AVERAGE(I26:I27)</f>
+        <v>0.35124898845084079</v>
+      </c>
+      <c r="O26" s="17">
+        <f>AVERAGE(J26:J27)</f>
+        <v>2131.6417367546246</v>
+      </c>
+      <c r="P26" s="17">
+        <f>AVERAGE(K26:K27)</f>
+        <v>1381.5473104947814</v>
+      </c>
+      <c r="R26" s="17">
+        <f>SUM(O26:P26)</f>
+        <v>3513.189047249406</v>
+      </c>
+      <c r="S26" s="17">
+        <f>SUM(O40:P40)</f>
+        <v>3459.5092267935465</v>
+      </c>
+    </row>
+    <row r="27" spans="1:19" ht="15" x14ac:dyDescent="0.25">
+      <c r="A27" s="22">
+        <v>8</v>
+      </c>
+      <c r="B27" s="22"/>
+      <c r="C27" s="22">
+        <v>31</v>
+      </c>
+      <c r="D27" s="22">
+        <v>17.72</v>
+      </c>
+      <c r="E27" s="22">
+        <f>1236-64.82</f>
+        <v>1171.18</v>
+      </c>
+      <c r="F27" s="22">
+        <f>655.58-23.95</f>
+        <v>631.63</v>
+      </c>
+      <c r="G27" s="22">
+        <f>477.45-64.82</f>
+        <v>412.63</v>
+      </c>
+      <c r="H27" s="21">
+        <f>F27/E27</f>
+        <v>0.53931078058026949</v>
+      </c>
+      <c r="I27" s="20">
+        <f>G27/E27</f>
+        <v>0.35231988251165491</v>
+      </c>
+      <c r="J27" s="18">
+        <f>D27*H27/44*10000</f>
+        <v>2171.9515981550853</v>
+      </c>
+      <c r="K27" s="18">
+        <f>I27*D27/44*10000</f>
+        <v>1418.8882541151193</v>
+      </c>
+      <c r="L27" s="18">
+        <f>D27/44*10000*0.35</f>
+        <v>1409.5454545454543</v>
+      </c>
+      <c r="N27" s="19"/>
+      <c r="R27" s="17"/>
+      <c r="S27" s="17">
+        <f>SUM(O42:P42)</f>
+        <v>3145.8222744862273</v>
+      </c>
+    </row>
+    <row r="28" spans="1:19" ht="15" x14ac:dyDescent="0.25">
+      <c r="A28" s="22">
+        <v>9</v>
+      </c>
+      <c r="B28" s="22">
+        <v>32</v>
+      </c>
+      <c r="C28" s="22"/>
+      <c r="D28" s="22">
+        <v>18.47</v>
+      </c>
+      <c r="E28" s="22">
+        <f>908.14-64.82</f>
+        <v>843.31999999999994</v>
+      </c>
+      <c r="F28" s="22">
+        <f>496.42-23.95</f>
+        <v>472.47</v>
+      </c>
+      <c r="G28" s="22">
+        <f>363.88-64.82</f>
+        <v>299.06</v>
+      </c>
+      <c r="H28" s="21">
+        <f>F28/E28</f>
+        <v>0.56024996442631514</v>
+      </c>
+      <c r="I28" s="20">
+        <f>G28/E28</f>
+        <v>0.3546222074657307</v>
+      </c>
+      <c r="J28" s="18">
+        <f>D28*H28/44*10000</f>
+        <v>2351.7765552168275</v>
+      </c>
+      <c r="K28" s="18">
+        <f>I28*D28/44*10000</f>
+        <v>1488.6073117936467</v>
+      </c>
+      <c r="L28" s="18">
+        <f>D28/44*10000*0.35</f>
+        <v>1469.204545454545</v>
+      </c>
+      <c r="M28" s="15">
+        <f>A28</f>
+        <v>9</v>
+      </c>
+      <c r="N28" s="19">
+        <f>AVERAGE(I28:I29)</f>
+        <v>0.36078334098797954</v>
+      </c>
+      <c r="O28" s="17">
+        <f>AVERAGE(J28:J29)</f>
+        <v>2408.2442734363758</v>
+      </c>
+      <c r="P28" s="17">
+        <f>AVERAGE(K28:K29)</f>
+        <v>1560.3381293246835</v>
+      </c>
+      <c r="R28" s="17">
+        <f>SUM(O28:P28)</f>
+        <v>3968.5824027610593</v>
+      </c>
+    </row>
+    <row r="29" spans="1:19" ht="15" x14ac:dyDescent="0.25">
+      <c r="A29" s="22">
+        <v>9</v>
+      </c>
+      <c r="B29" s="22"/>
+      <c r="C29" s="22">
+        <v>36</v>
+      </c>
+      <c r="D29" s="22">
+        <v>19.57</v>
+      </c>
+      <c r="E29" s="22">
+        <f>988.72-64.82</f>
+        <v>923.90000000000009</v>
+      </c>
+      <c r="F29" s="22">
+        <f>535.93-23.95</f>
+        <v>511.97999999999996</v>
+      </c>
+      <c r="G29" s="22">
+        <f>403.85-64.83</f>
+        <v>339.02000000000004</v>
+      </c>
+      <c r="H29" s="21">
+        <f>F29/E29</f>
+        <v>0.55415088213010055</v>
+      </c>
+      <c r="I29" s="20">
+        <f>G29/E29</f>
+        <v>0.36694447451022838</v>
+      </c>
+      <c r="J29" s="18">
+        <f>D29*H29/44*10000</f>
+        <v>2464.7119916559245</v>
+      </c>
+      <c r="K29" s="18">
+        <f>I29*D29/44*10000</f>
+        <v>1632.0689468557202</v>
+      </c>
+      <c r="L29" s="18">
+        <f>D29/44*10000*0.35</f>
+        <v>1556.7045454545455</v>
+      </c>
+      <c r="N29" s="19"/>
+      <c r="R29" s="17"/>
+    </row>
+    <row r="30" spans="1:19" ht="15" x14ac:dyDescent="0.25">
+      <c r="A30" s="22">
+        <v>10</v>
+      </c>
+      <c r="B30" s="22">
+        <v>33</v>
+      </c>
+      <c r="C30" s="22"/>
+      <c r="D30" s="22">
+        <v>15.86</v>
+      </c>
+      <c r="E30" s="22">
+        <f>890.96-64.82</f>
+        <v>826.1400000000001</v>
+      </c>
+      <c r="F30" s="22">
+        <f>465.39-23.95</f>
+        <v>441.44</v>
+      </c>
+      <c r="G30" s="22">
+        <f>338.03-64.82</f>
+        <v>273.20999999999998</v>
+      </c>
+      <c r="H30" s="21">
+        <f>F30/E30</f>
+        <v>0.5343404265620838</v>
+      </c>
+      <c r="I30" s="20">
+        <f>G30/E30</f>
+        <v>0.33070665988815451</v>
+      </c>
+      <c r="J30" s="18">
+        <f>D30*H30/44*10000</f>
+        <v>1926.0543557442384</v>
+      </c>
+      <c r="K30" s="18">
+        <f>I30*D30/44*10000</f>
+        <v>1192.0471876877571</v>
+      </c>
+      <c r="L30" s="18">
+        <f>D30/44*10000*0.35</f>
+        <v>1261.5909090909088</v>
+      </c>
+      <c r="M30" s="15">
+        <f>A30</f>
+        <v>10</v>
+      </c>
+      <c r="N30" s="19">
+        <f>AVERAGE(I30:I31)</f>
+        <v>0.33925981708265374</v>
+      </c>
+      <c r="O30" s="17">
+        <f>AVERAGE(J30:J31)</f>
+        <v>2032.5276302595571</v>
+      </c>
+      <c r="P30" s="17">
+        <f>AVERAGE(K30:K31)</f>
+        <v>1269.9112315058624</v>
+      </c>
+      <c r="R30" s="17">
+        <f>SUM(O30:P30)</f>
+        <v>3302.4388617654195</v>
+      </c>
+      <c r="S30" s="17">
+        <f>AVERAGE(S12,S18,S23,S25)</f>
+        <v>3133.976785997118</v>
+      </c>
+    </row>
+    <row r="31" spans="1:19" ht="15" x14ac:dyDescent="0.25">
+      <c r="A31" s="22">
+        <v>10</v>
+      </c>
+      <c r="B31" s="22"/>
+      <c r="C31" s="22">
+        <v>37</v>
+      </c>
+      <c r="D31" s="22">
+        <v>17.05</v>
+      </c>
+      <c r="E31" s="22">
+        <f>1092.7-64.82</f>
+        <v>1027.8800000000001</v>
+      </c>
+      <c r="F31" s="22">
+        <f>591.34-23.95</f>
+        <v>567.39</v>
+      </c>
+      <c r="G31" s="22">
+        <f>422.33-64.82</f>
+        <v>357.51</v>
+      </c>
+      <c r="H31" s="21">
+        <f>F31/E31</f>
+        <v>0.55200023349029059</v>
+      </c>
+      <c r="I31" s="20">
+        <f>G31/E31</f>
+        <v>0.34781297427715291</v>
+      </c>
+      <c r="J31" s="18">
+        <f>D31*H31/44*10000</f>
+        <v>2139.0009047748758</v>
+      </c>
+      <c r="K31" s="18">
+        <f>I31*D31/44*10000</f>
+        <v>1347.7752753239677</v>
+      </c>
+      <c r="L31" s="18">
+        <f>D31/44*10000*0.35</f>
+        <v>1356.25</v>
+      </c>
+      <c r="N31" s="19"/>
+      <c r="R31" s="17"/>
+      <c r="S31" s="17">
+        <f>AVERAGE(S13,S19,S20,S26)</f>
+        <v>3508.2480031603623</v>
+      </c>
+    </row>
+    <row r="32" spans="1:19" ht="15" x14ac:dyDescent="0.25">
+      <c r="A32" s="22">
+        <v>11</v>
+      </c>
+      <c r="B32" s="22">
+        <v>34</v>
+      </c>
+      <c r="C32" s="22"/>
+      <c r="D32" s="22">
+        <v>17.420000000000002</v>
+      </c>
+      <c r="E32" s="22">
+        <f>942.5-64.82</f>
+        <v>877.68000000000006</v>
+      </c>
+      <c r="F32" s="22">
+        <f>476.37-23.95</f>
+        <v>452.42</v>
+      </c>
+      <c r="G32" s="22">
+        <f>361.75-64.82</f>
+        <v>296.93</v>
+      </c>
+      <c r="H32" s="21">
+        <f>F32/E32</f>
+        <v>0.51547260960714614</v>
+      </c>
+      <c r="I32" s="20">
+        <f>G32/E32</f>
+        <v>0.3383123689727463</v>
+      </c>
+      <c r="J32" s="18">
+        <f>D32*H32/44*10000</f>
+        <v>2040.8029225810199</v>
+      </c>
+      <c r="K32" s="18">
+        <f>I32*D32/44*10000</f>
+        <v>1339.4094244330092</v>
+      </c>
+      <c r="L32" s="18">
+        <f>D32/44*10000*0.35</f>
+        <v>1385.6818181818182</v>
+      </c>
+      <c r="M32" s="15">
+        <f>A32</f>
+        <v>11</v>
+      </c>
+      <c r="N32" s="19">
+        <f>AVERAGE(I32:I33)</f>
+        <v>0.33793086126890781</v>
+      </c>
+      <c r="O32" s="17">
+        <f>AVERAGE(J32:J33)</f>
+        <v>2071.6193330873666</v>
+      </c>
+      <c r="P32" s="17">
+        <f>AVERAGE(K32:K33)</f>
+        <v>1358.9958353488107</v>
+      </c>
+      <c r="R32" s="17">
+        <f>SUM(O32:P32)</f>
+        <v>3430.6151684361776</v>
+      </c>
+      <c r="S32" s="17">
+        <f>AVERAGE(S14,S16,S21,S27)</f>
+        <v>3249.9760493613717</v>
+      </c>
+    </row>
+    <row r="33" spans="1:19" ht="15" x14ac:dyDescent="0.25">
+      <c r="A33" s="22">
+        <v>11</v>
+      </c>
+      <c r="B33" s="22"/>
+      <c r="C33" s="22">
+        <v>38</v>
+      </c>
+      <c r="D33" s="22">
+        <v>17.97</v>
+      </c>
+      <c r="E33" s="22">
+        <f>1098.18-64.82</f>
+        <v>1033.3600000000001</v>
+      </c>
+      <c r="F33" s="22">
+        <f>555.91-23.95</f>
+        <v>531.95999999999992</v>
+      </c>
+      <c r="G33" s="22">
+        <f>413.63-64.82</f>
+        <v>348.81</v>
+      </c>
+      <c r="H33" s="21">
+        <f>F33/E33</f>
+        <v>0.51478671518154362</v>
+      </c>
+      <c r="I33" s="20">
+        <f>G33/E33</f>
+        <v>0.33754935356506927</v>
+      </c>
+      <c r="J33" s="18">
+        <f>D33*H33/44*10000</f>
+        <v>2102.4357435937131</v>
+      </c>
+      <c r="K33" s="18">
+        <f>I33*D33/44*10000</f>
+        <v>1378.5822462646122</v>
+      </c>
+      <c r="L33" s="18">
+        <f>D33/44*10000*0.35</f>
+        <v>1429.431818181818</v>
+      </c>
+      <c r="N33" s="19"/>
+      <c r="R33" s="17"/>
+      <c r="S33" s="17">
+        <f>AVERAGE(S15,S17,S22,S24)</f>
+        <v>3478.5675069323233</v>
+      </c>
+    </row>
+    <row r="34" spans="1:19" ht="15" x14ac:dyDescent="0.25">
+      <c r="A34" s="22">
+        <v>12</v>
+      </c>
+      <c r="B34" s="22">
+        <v>35</v>
+      </c>
+      <c r="C34" s="22"/>
+      <c r="D34" s="22">
+        <v>14.6</v>
+      </c>
+      <c r="E34" s="22">
+        <f>1190.48-64.82</f>
+        <v>1125.6600000000001</v>
+      </c>
+      <c r="F34" s="22">
+        <f>646.42-23.95</f>
+        <v>622.46999999999991</v>
+      </c>
+      <c r="G34" s="22">
+        <f>427.6-64.82</f>
+        <v>362.78000000000003</v>
+      </c>
+      <c r="H34" s="21">
+        <f>F34/E34</f>
+        <v>0.5529822504130909</v>
+      </c>
+      <c r="I34" s="20">
+        <f>G34/E34</f>
+        <v>0.32228203898157526</v>
+      </c>
+      <c r="J34" s="18">
+        <f>D34*H34/44*10000</f>
+        <v>1834.8956490979831</v>
+      </c>
+      <c r="K34" s="18">
+        <f>I34*D34/44*10000</f>
+        <v>1069.390402075227</v>
+      </c>
+      <c r="L34" s="18">
+        <f>D34/44*10000*0.35</f>
+        <v>1161.3636363636363</v>
+      </c>
+      <c r="M34" s="15">
+        <f>A34</f>
+        <v>12</v>
+      </c>
+      <c r="N34" s="19">
+        <f>AVERAGE(I34:I35)</f>
+        <v>0.33239072307153222</v>
+      </c>
+      <c r="O34" s="17">
+        <f>AVERAGE(J34:J35)</f>
+        <v>2009.7960902268751</v>
+      </c>
+      <c r="P34" s="17">
+        <f>AVERAGE(K34:K35)</f>
+        <v>1198.6770062847731</v>
+      </c>
+      <c r="R34" s="17">
+        <f>SUM(O34:P34)</f>
+        <v>3208.4730965116482</v>
+      </c>
+    </row>
+    <row r="35" spans="1:19" ht="15" x14ac:dyDescent="0.25">
+      <c r="A35" s="22">
+        <v>12</v>
+      </c>
+      <c r="B35" s="22"/>
+      <c r="C35" s="22">
+        <v>39</v>
+      </c>
+      <c r="D35" s="22">
+        <v>17.059999999999999</v>
+      </c>
+      <c r="E35" s="22">
+        <f>1119.08-64.83</f>
+        <v>1054.25</v>
+      </c>
+      <c r="F35" s="22">
+        <f>617.98-23.95</f>
+        <v>594.03</v>
+      </c>
+      <c r="G35" s="22">
+        <f>425.9-64.82</f>
+        <v>361.08</v>
+      </c>
+      <c r="H35" s="21">
+        <f>F35/E35</f>
+        <v>0.56346217690301159</v>
+      </c>
+      <c r="I35" s="20">
+        <f>G35/E35</f>
+        <v>0.34249940716148919</v>
+      </c>
+      <c r="J35" s="18">
+        <f>D35*H35/44*10000</f>
+        <v>2184.6965313557671</v>
+      </c>
+      <c r="K35" s="18">
+        <f>I35*D35/44*10000</f>
+        <v>1327.9636104943193</v>
+      </c>
+      <c r="L35" s="18">
+        <f>D35/44*10000*0.35</f>
+        <v>1357.0454545454543</v>
+      </c>
+      <c r="N35" s="19"/>
+      <c r="R35" s="17"/>
+    </row>
+    <row r="36" spans="1:19" ht="15" x14ac:dyDescent="0.25">
+      <c r="A36" s="22">
+        <v>13</v>
+      </c>
+      <c r="B36" s="22">
+        <v>40</v>
+      </c>
+      <c r="C36" s="22"/>
+      <c r="D36" s="22">
+        <f>15.64-0.51</f>
+        <v>15.13</v>
+      </c>
+      <c r="E36" s="22">
+        <f>1036.2-64.82</f>
+        <v>971.38000000000011</v>
+      </c>
+      <c r="F36" s="22">
+        <f>561.56-23.95</f>
+        <v>537.6099999999999</v>
+      </c>
+      <c r="G36" s="22">
+        <f>411.63-64.82</f>
+        <v>346.81</v>
+      </c>
+      <c r="H36" s="21">
+        <f>F36/E36</f>
+        <v>0.55344973131009478</v>
+      </c>
+      <c r="I36" s="20">
+        <f>G36/E36</f>
+        <v>0.35702814552492329</v>
+      </c>
+      <c r="J36" s="18">
+        <f>D36*H36/44*10000</f>
+        <v>1903.1123715276669</v>
+      </c>
+      <c r="K36" s="18">
+        <f>I36*D36/44*10000</f>
+        <v>1227.6899640436568</v>
+      </c>
+      <c r="L36" s="18">
+        <f>D36/44*10000*0.35</f>
+        <v>1203.5227272727273</v>
+      </c>
+      <c r="M36" s="15">
+        <f>A36</f>
+        <v>13</v>
+      </c>
+      <c r="N36" s="19">
+        <f>AVERAGE(I36:I37)</f>
+        <v>0.35391275900522762</v>
+      </c>
+      <c r="O36" s="17">
+        <f>AVERAGE(J36:J37)</f>
+        <v>1941.4721664550191</v>
+      </c>
+      <c r="P36" s="17">
+        <f>AVERAGE(K36:K37)</f>
+        <v>1240.0980185840676</v>
+      </c>
+      <c r="R36" s="17">
+        <f>SUM(O36:P36)</f>
+        <v>3181.5701850390869</v>
+      </c>
+    </row>
+    <row r="37" spans="1:19" ht="15" x14ac:dyDescent="0.25">
+      <c r="A37" s="22">
+        <v>13</v>
+      </c>
+      <c r="B37" s="22"/>
+      <c r="C37" s="22">
+        <v>41</v>
+      </c>
+      <c r="D37" s="26">
+        <f>16.22-0.51</f>
+        <v>15.709999999999999</v>
+      </c>
+      <c r="E37" s="22">
+        <f>1139.6-64.82</f>
+        <v>1074.78</v>
+      </c>
+      <c r="F37" s="22">
+        <f>619.92-23.95</f>
+        <v>595.96999999999991</v>
+      </c>
+      <c r="G37" s="22">
+        <f>441.86-64.83</f>
+        <v>377.03000000000003</v>
+      </c>
+      <c r="H37" s="21">
+        <f>F37/E37</f>
+        <v>0.55450417759913651</v>
+      </c>
+      <c r="I37" s="20">
+        <f>G37/E37</f>
+        <v>0.35079737248553194</v>
+      </c>
+      <c r="J37" s="18">
+        <f>D37*H37/44*10000</f>
+        <v>1979.8319613823712</v>
+      </c>
+      <c r="K37" s="18">
+        <f>I37*D37/44*10000</f>
+        <v>1252.5060731244787</v>
+      </c>
+      <c r="L37" s="18">
+        <f>D37/44*10000*0.35</f>
+        <v>1249.6590909090908</v>
+      </c>
+      <c r="N37" s="19"/>
+      <c r="R37" s="17"/>
+    </row>
+    <row r="38" spans="1:19" ht="15" x14ac:dyDescent="0.25">
+      <c r="A38" s="22">
+        <v>14</v>
+      </c>
+      <c r="B38" s="22">
+        <v>42</v>
+      </c>
+      <c r="C38" s="22"/>
+      <c r="D38" s="22">
+        <f>15.17-0.51</f>
+        <v>14.66</v>
+      </c>
+      <c r="E38" s="22">
+        <f>1253.35-64.82</f>
+        <v>1188.53</v>
+      </c>
+      <c r="F38" s="22">
+        <f>690.78-23.95</f>
+        <v>666.82999999999993</v>
+      </c>
+      <c r="G38" s="22">
+        <f>484.16-64.82</f>
+        <v>419.34000000000003</v>
+      </c>
+      <c r="H38" s="21">
+        <f>F38/E38</f>
+        <v>0.56105441175233262</v>
+      </c>
+      <c r="I38" s="20">
+        <f>G38/E38</f>
+        <v>0.35282239404979265</v>
+      </c>
+      <c r="J38" s="18">
+        <f>D38*H38/44*10000</f>
+        <v>1869.3312900657265</v>
+      </c>
+      <c r="K38" s="18">
+        <f>I38*D38/44*10000</f>
+        <v>1175.5400674477182</v>
+      </c>
+      <c r="L38" s="18">
+        <f>D38/44*10000*0.35</f>
+        <v>1166.1363636363635</v>
+      </c>
+      <c r="M38" s="15">
+        <f>A38</f>
+        <v>14</v>
+      </c>
+      <c r="N38" s="19">
+        <f>AVERAGE(I38:I39)</f>
+        <v>0.34247880108486461</v>
+      </c>
+      <c r="O38" s="17">
+        <f>AVERAGE(J38:J39)</f>
+        <v>1906.3692169754004</v>
+      </c>
+      <c r="P38" s="17">
+        <f>AVERAGE(K38:K39)</f>
+        <v>1190.5199511869714</v>
+      </c>
+      <c r="R38" s="17">
+        <f>SUM(O38:P38)</f>
+        <v>3096.8891681623718</v>
+      </c>
+    </row>
+    <row r="39" spans="1:19" ht="15" x14ac:dyDescent="0.25">
+      <c r="A39" s="22">
+        <v>14</v>
+      </c>
+      <c r="B39" s="22"/>
+      <c r="C39" s="22">
+        <v>43</v>
+      </c>
+      <c r="D39" s="22">
+        <f>16.48-0.51</f>
+        <v>15.97</v>
+      </c>
+      <c r="E39" s="22">
+        <f>1138.72-64.82</f>
+        <v>1073.9000000000001</v>
+      </c>
+      <c r="F39" s="22">
+        <f>598.96-23.95</f>
+        <v>575.01</v>
+      </c>
+      <c r="G39" s="22">
+        <f>421.5-64.82</f>
+        <v>356.68</v>
+      </c>
+      <c r="H39" s="21">
+        <f>F39/E39</f>
+        <v>0.53544091628643253</v>
+      </c>
+      <c r="I39" s="20">
+        <f>G39/E39</f>
+        <v>0.33213520811993663</v>
+      </c>
+      <c r="J39" s="18">
+        <f>D39*H39/44*10000</f>
+        <v>1943.4071438850744</v>
+      </c>
+      <c r="K39" s="18">
+        <f>I39*D39/44*10000</f>
+        <v>1205.4998349262246</v>
+      </c>
+      <c r="L39" s="18">
+        <f>D39/44*10000*0.35</f>
+        <v>1270.3409090909092</v>
+      </c>
+      <c r="N39" s="19"/>
+      <c r="R39" s="17"/>
+    </row>
+    <row r="40" spans="1:19" ht="15" x14ac:dyDescent="0.25">
+      <c r="A40" s="22">
+        <v>15</v>
+      </c>
+      <c r="B40" s="22">
+        <v>44</v>
+      </c>
+      <c r="C40" s="22"/>
+      <c r="D40" s="22">
+        <f>17.69-0.51</f>
+        <v>17.18</v>
+      </c>
+      <c r="E40" s="22">
+        <f>969.7-64.83</f>
+        <v>904.87</v>
+      </c>
+      <c r="F40" s="22">
+        <f>527.95-23.95</f>
+        <v>504.00000000000006</v>
+      </c>
+      <c r="G40" s="22">
+        <f>392.84-64.82</f>
+        <v>328.02</v>
+      </c>
+      <c r="H40" s="21">
+        <f>F40/E40</f>
+        <v>0.55698608639915137</v>
+      </c>
+      <c r="I40" s="20">
+        <f>G40/E40</f>
+        <v>0.36250511123144757</v>
+      </c>
+      <c r="J40" s="18">
+        <f>D40*H40/44*10000</f>
+        <v>2174.7774918948685</v>
+      </c>
+      <c r="K40" s="18">
+        <f>I40*D40/44*10000</f>
+        <v>1415.417684308243</v>
+      </c>
+      <c r="L40" s="18">
+        <f>D40/44*10000*0.35</f>
+        <v>1366.590909090909</v>
+      </c>
+      <c r="M40" s="15">
+        <f>A40</f>
+        <v>15</v>
+      </c>
+      <c r="N40" s="19">
+        <f>AVERAGE(I40:I41)</f>
+        <v>0.36188241051825931</v>
+      </c>
+      <c r="O40" s="17">
+        <f>AVERAGE(J40:J41)</f>
+        <v>2096.1961158227223</v>
+      </c>
+      <c r="P40" s="17">
+        <f>AVERAGE(K40:K41)</f>
+        <v>1363.3131109708243</v>
+      </c>
+      <c r="R40" s="17">
+        <f>SUM(O40:P40)</f>
+        <v>3459.5092267935465</v>
+      </c>
+    </row>
+    <row r="41" spans="1:19" ht="15" x14ac:dyDescent="0.25">
+      <c r="A41" s="22">
+        <v>15</v>
+      </c>
+      <c r="B41" s="22"/>
+      <c r="C41" s="22">
+        <v>45</v>
+      </c>
+      <c r="D41" s="22">
+        <f>16.48-0.51</f>
+        <v>15.97</v>
+      </c>
+      <c r="E41" s="22">
+        <f>1156.5-64.82</f>
+        <v>1091.68</v>
+      </c>
+      <c r="F41" s="22">
+        <f>630.8-23.95</f>
+        <v>606.84999999999991</v>
+      </c>
+      <c r="G41" s="22">
+        <f>459.2-64.82</f>
+        <v>394.38</v>
+      </c>
+      <c r="H41" s="21">
+        <f>F41/E41</f>
+        <v>0.55588634031950745</v>
+      </c>
+      <c r="I41" s="20">
+        <f>G41/E41</f>
+        <v>0.36125970980507105</v>
+      </c>
+      <c r="J41" s="18">
+        <f>D41*H41/44*10000</f>
+        <v>2017.6147397505761</v>
+      </c>
+      <c r="K41" s="18">
+        <f>I41*D41/44*10000</f>
+        <v>1311.2085376334057</v>
+      </c>
+      <c r="L41" s="18">
+        <f>D41/44*10000*0.35</f>
+        <v>1270.3409090909092</v>
+      </c>
+      <c r="N41" s="19"/>
+      <c r="R41" s="17"/>
+    </row>
+    <row r="42" spans="1:19" ht="15" x14ac:dyDescent="0.25">
+      <c r="A42" s="25">
+        <v>16</v>
+      </c>
+      <c r="B42" s="25">
+        <v>46</v>
+      </c>
+      <c r="C42" s="25"/>
+      <c r="D42" s="25">
+        <f>16.53-0.51</f>
+        <v>16.02</v>
+      </c>
+      <c r="E42" s="25">
+        <f>981.45-64.82</f>
+        <v>916.63000000000011</v>
+      </c>
+      <c r="F42" s="25">
+        <f>609.62-23.95</f>
+        <v>585.66999999999996</v>
+      </c>
+      <c r="G42" s="25">
+        <f>219.49-64.82</f>
+        <v>154.67000000000002</v>
+      </c>
+      <c r="H42" s="24">
+        <f>F42/E42</f>
+        <v>0.63893828480411929</v>
+      </c>
+      <c r="I42" s="24">
+        <f>G42/E42</f>
+        <v>0.16873765859725298</v>
+      </c>
+      <c r="J42" s="23">
+        <f>D42*H42/44*10000</f>
+        <v>2326.3162096731794</v>
+      </c>
+      <c r="K42" s="23">
+        <f>I42*D42/44*10000</f>
+        <v>614.35847516545289</v>
+      </c>
+      <c r="L42" s="18">
+        <f>D42/44*10000*0.35</f>
+        <v>1274.3181818181815</v>
+      </c>
+      <c r="M42" s="15">
+        <f>A42</f>
+        <v>16</v>
+      </c>
+      <c r="N42" s="19">
+        <f>I43</f>
+        <v>0.32893374271024467</v>
+      </c>
+      <c r="O42" s="17">
+        <f>J43</f>
+        <v>1954.1850338495683</v>
+      </c>
+      <c r="P42" s="17">
+        <f>K43</f>
+        <v>1191.637240636659</v>
+      </c>
+      <c r="R42" s="17">
+        <f>SUM(O42:P42)</f>
+        <v>3145.8222744862273</v>
+      </c>
+    </row>
+    <row r="43" spans="1:19" ht="15" x14ac:dyDescent="0.25">
+      <c r="A43" s="22">
+        <v>16</v>
+      </c>
+      <c r="B43" s="22"/>
+      <c r="C43" s="22">
+        <v>47</v>
+      </c>
+      <c r="D43" s="22">
+        <f>16.45-0.51</f>
+        <v>15.94</v>
+      </c>
+      <c r="E43" s="22">
+        <f>1165.68-64.82</f>
+        <v>1100.8600000000001</v>
+      </c>
+      <c r="F43" s="22">
+        <f>617.78-23.95</f>
+        <v>593.82999999999993</v>
+      </c>
+      <c r="G43" s="22">
+        <f>426.93-64.82</f>
+        <v>362.11</v>
+      </c>
+      <c r="H43" s="21">
+        <f>F43/E43</f>
+        <v>0.53942372327089716</v>
+      </c>
+      <c r="I43" s="20">
+        <f>G43/E43</f>
+        <v>0.32893374271024467</v>
+      </c>
+      <c r="J43" s="18">
+        <f>D43*H43/44*10000</f>
+        <v>1954.1850338495683</v>
+      </c>
+      <c r="K43" s="18">
+        <f>I43*D43/44*10000</f>
+        <v>1191.637240636659</v>
+      </c>
+      <c r="L43" s="18">
+        <f>D43/44*10000*0.35</f>
+        <v>1267.9545454545453</v>
+      </c>
+    </row>
+    <row r="44" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A44" s="16"/>
+      <c r="B44" s="16"/>
+      <c r="C44" s="16"/>
+      <c r="D44" s="16"/>
+      <c r="E44" s="16"/>
+      <c r="F44" s="16"/>
+      <c r="G44" s="16"/>
+    </row>
+    <row r="45" spans="1:19" ht="15" x14ac:dyDescent="0.25">
+      <c r="A45" s="16"/>
+      <c r="B45" s="16"/>
+      <c r="C45" s="16"/>
+      <c r="D45" s="16"/>
+      <c r="E45" s="16"/>
+      <c r="F45" s="16"/>
+      <c r="G45" s="16" t="s">
+        <v>134</v>
+      </c>
+      <c r="H45" s="19">
+        <f>AVERAGE(H12:H41,H43)</f>
+        <v>0.54645975160944793</v>
+      </c>
+      <c r="I45" s="19">
+        <f>AVERAGE(I12:I41,I43)</f>
+        <v>0.34705762526716072</v>
+      </c>
+      <c r="J45" s="18">
+        <f>AVERAGE(J12:J41,J43)</f>
+        <v>2047.5817189474667</v>
+      </c>
+      <c r="K45" s="18">
+        <f>AVERAGE(K12:K41,K43)</f>
+        <v>1301.4610065081201</v>
+      </c>
+      <c r="Q45" s="15" t="s">
+        <v>133</v>
+      </c>
+      <c r="R45" s="17">
+        <f>AVERAGE(R12,R24,R34,R38)</f>
+        <v>3133.976785997118</v>
+      </c>
+    </row>
+    <row r="46" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A46" s="16"/>
+      <c r="B46" s="16"/>
+      <c r="C46" s="16"/>
+      <c r="D46" s="16"/>
+      <c r="E46" s="16"/>
+      <c r="F46" s="16"/>
+      <c r="G46" s="16"/>
+      <c r="Q46" s="15" t="s">
+        <v>132</v>
+      </c>
+      <c r="R46" s="17">
+        <f>AVERAGE(R14,R26,R28,R40)</f>
+        <v>3508.2480031603623</v>
+      </c>
+    </row>
+    <row r="47" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A47" s="16"/>
+      <c r="B47" s="16"/>
+      <c r="C47" s="16"/>
+      <c r="D47" s="16"/>
+      <c r="E47" s="16"/>
+      <c r="F47" s="16"/>
+      <c r="G47" s="16"/>
+      <c r="Q47" s="15" t="s">
+        <v>131</v>
+      </c>
+      <c r="R47" s="17">
+        <f>AVERAGE(R16,R20,R30,R42)</f>
+        <v>3249.9760493613717</v>
+      </c>
+    </row>
+    <row r="48" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A48" s="16"/>
+      <c r="B48" s="16"/>
+      <c r="C48" s="16"/>
+      <c r="D48" s="16"/>
+      <c r="E48" s="16"/>
+      <c r="F48" s="16"/>
+      <c r="G48" s="16"/>
+      <c r="Q48" s="15" t="s">
+        <v>130</v>
+      </c>
+      <c r="R48" s="17">
+        <f>AVERAGE(R18,R22,R32,R36)</f>
+        <v>3478.5675069323233</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A49" s="16"/>
+      <c r="B49" s="16"/>
+      <c r="C49" s="16"/>
+      <c r="D49" s="16"/>
+      <c r="E49" s="16"/>
+      <c r="F49" s="16"/>
+      <c r="G49" s="16"/>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A50" s="16"/>
+      <c r="B50" s="16"/>
+      <c r="C50" s="16"/>
+      <c r="D50" s="16"/>
+      <c r="E50" s="16"/>
+      <c r="F50" s="16"/>
+      <c r="G50" s="16"/>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A51" s="16"/>
+      <c r="B51" s="16"/>
+      <c r="C51" s="16"/>
+      <c r="D51" s="16"/>
+      <c r="E51" s="16"/>
+      <c r="F51" s="16"/>
+      <c r="G51" s="16"/>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A52" s="16"/>
+      <c r="B52" s="16"/>
+      <c r="C52" s="16"/>
+      <c r="D52" s="16"/>
+      <c r="E52" s="16"/>
+      <c r="F52" s="16"/>
+      <c r="G52" s="16"/>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A53" s="16"/>
+      <c r="B53" s="16"/>
+      <c r="C53" s="16"/>
+      <c r="D53" s="16"/>
+      <c r="E53" s="16"/>
+      <c r="F53" s="16"/>
+      <c r="G53" s="16"/>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A54" s="16"/>
+      <c r="B54" s="16"/>
+      <c r="C54" s="16"/>
+      <c r="D54" s="16"/>
+      <c r="E54" s="16"/>
+      <c r="F54" s="16"/>
+      <c r="G54" s="16"/>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A55" s="16"/>
+      <c r="B55" s="16"/>
+      <c r="C55" s="16"/>
+      <c r="D55" s="16"/>
+      <c r="E55" s="16"/>
+      <c r="F55" s="16"/>
+      <c r="G55" s="16"/>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A56" s="16"/>
+      <c r="B56" s="16"/>
+      <c r="C56" s="16"/>
+      <c r="D56" s="16"/>
+      <c r="E56" s="16"/>
+      <c r="F56" s="16"/>
+      <c r="G56" s="16"/>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A57" s="16"/>
+      <c r="B57" s="16"/>
+      <c r="C57" s="16"/>
+      <c r="D57" s="16"/>
+      <c r="E57" s="16"/>
+      <c r="F57" s="16"/>
+      <c r="G57" s="16"/>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A58" s="16"/>
+      <c r="B58" s="16"/>
+      <c r="C58" s="16"/>
+      <c r="D58" s="16"/>
+      <c r="E58" s="16"/>
+      <c r="F58" s="16"/>
+      <c r="G58" s="16"/>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A59" s="16"/>
+      <c r="B59" s="16"/>
+      <c r="C59" s="16"/>
+      <c r="D59" s="16"/>
+      <c r="E59" s="16"/>
+      <c r="F59" s="16"/>
+      <c r="G59" s="16"/>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A60" s="16"/>
+      <c r="B60" s="16"/>
+      <c r="C60" s="16"/>
+      <c r="D60" s="16"/>
+      <c r="E60" s="16"/>
+      <c r="F60" s="16"/>
+      <c r="G60" s="16"/>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A61" s="16"/>
+      <c r="B61" s="16"/>
+      <c r="C61" s="16"/>
+      <c r="D61" s="16"/>
+      <c r="E61" s="16"/>
+      <c r="F61" s="16"/>
+      <c r="G61" s="16"/>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A62" s="16"/>
+      <c r="B62" s="16"/>
+      <c r="C62" s="16"/>
+      <c r="D62" s="16"/>
+      <c r="E62" s="16"/>
+      <c r="F62" s="16"/>
+      <c r="G62" s="16"/>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A63" s="16"/>
+      <c r="B63" s="16"/>
+      <c r="C63" s="16"/>
+      <c r="D63" s="16"/>
+      <c r="E63" s="16"/>
+      <c r="F63" s="16"/>
+      <c r="G63" s="16"/>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A64" s="16"/>
+      <c r="B64" s="16"/>
+      <c r="C64" s="16"/>
+      <c r="D64" s="16"/>
+      <c r="E64" s="16"/>
+      <c r="F64" s="16"/>
+      <c r="G64" s="16"/>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A65" s="16"/>
+      <c r="B65" s="16"/>
+      <c r="C65" s="16"/>
+      <c r="D65" s="16"/>
+      <c r="E65" s="16"/>
+      <c r="F65" s="16"/>
+      <c r="G65" s="16"/>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A66" s="16"/>
+      <c r="B66" s="16"/>
+      <c r="C66" s="16"/>
+      <c r="D66" s="16"/>
+      <c r="E66" s="16"/>
+      <c r="F66" s="16"/>
+      <c r="G66" s="16"/>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A67" s="16"/>
+      <c r="B67" s="16"/>
+      <c r="C67" s="16"/>
+      <c r="D67" s="16"/>
+      <c r="E67" s="16"/>
+      <c r="F67" s="16"/>
+      <c r="G67" s="16"/>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A68" s="16"/>
+      <c r="B68" s="16"/>
+      <c r="C68" s="16"/>
+      <c r="D68" s="16"/>
+      <c r="E68" s="16"/>
+      <c r="F68" s="16"/>
+      <c r="G68" s="16"/>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A69" s="16"/>
+      <c r="B69" s="16"/>
+      <c r="C69" s="16"/>
+      <c r="D69" s="16"/>
+      <c r="E69" s="16"/>
+      <c r="F69" s="16"/>
+      <c r="G69" s="16"/>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A70" s="16"/>
+      <c r="B70" s="16"/>
+      <c r="C70" s="16"/>
+      <c r="D70" s="16"/>
+      <c r="E70" s="16"/>
+      <c r="F70" s="16"/>
+      <c r="G70" s="16"/>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A71" s="16"/>
+      <c r="B71" s="16"/>
+      <c r="C71" s="16"/>
+      <c r="D71" s="16"/>
+      <c r="E71" s="16"/>
+      <c r="F71" s="16"/>
+      <c r="G71" s="16"/>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A72" s="16"/>
+      <c r="B72" s="16"/>
+      <c r="C72" s="16"/>
+      <c r="D72" s="16"/>
+      <c r="E72" s="16"/>
+      <c r="F72" s="16"/>
+      <c r="G72" s="16"/>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A73" s="16"/>
+      <c r="B73" s="16"/>
+      <c r="C73" s="16"/>
+      <c r="D73" s="16"/>
+      <c r="E73" s="16"/>
+      <c r="F73" s="16"/>
+      <c r="G73" s="16"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="M10:P10"/>
+    <mergeCell ref="H9:K9"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <headerFooter alignWithMargins="0"/>
+</worksheet>
 </file>
</xml_diff>